<commit_message>
Documentation and Figure Update
Work Journal Updates and I updated the correlation figure: I removed the model output notation in the figure because it is already in the text.
</commit_message>
<xml_diff>
--- a/Data Analysis/1_Data/ecological_multifunctionality_reduced.xlsx
+++ b/Data Analysis/1_Data/ecological_multifunctionality_reduced.xlsx
@@ -470,10 +470,10 @@
         <v>0.6159109451427114</v>
       </c>
       <c r="F2">
-        <v>152.379692735</v>
+        <v>175.9036689618518</v>
       </c>
       <c r="G2">
-        <v>0.341094719692547</v>
+        <v>0.3393615933846007</v>
       </c>
       <c r="H2">
         <v>11.83333333333333</v>
@@ -511,7 +511,7 @@
         <v>0.6467060369329617</v>
       </c>
       <c r="S2">
-        <v>0.5068951531028529</v>
+        <v>0.5066475636302892</v>
       </c>
     </row>
     <row r="3">
@@ -533,10 +533,10 @@
         <v>0.4765788354798875</v>
       </c>
       <c r="F3">
-        <v>275.3171712859375</v>
+        <v>316.0996166033333</v>
       </c>
       <c r="G3">
-        <v>0.7967257165554308</v>
+        <v>0.7846491592479132</v>
       </c>
       <c r="H3">
         <v>5.728813559322034</v>
@@ -574,7 +574,7 @@
         <v>0.7533089956157759</v>
       </c>
       <c r="S3">
-        <v>0.5452325353758232</v>
+        <v>0.5435073129033207</v>
       </c>
     </row>
     <row r="4">
@@ -596,10 +596,10 @@
         <v>0.5163091267147911</v>
       </c>
       <c r="F4">
-        <v>111.1061707528571</v>
+        <v>132.1994830808696</v>
       </c>
       <c r="G4">
-        <v>0.1881267542972417</v>
+        <v>0.2005492319977569</v>
       </c>
       <c r="H4">
         <v>6.186440677966102</v>
@@ -637,7 +637,7 @@
         <v>0.3618666178992232</v>
       </c>
       <c r="S4">
-        <v>0.4526777553726667</v>
+        <v>0.4544523950441689</v>
       </c>
     </row>
     <row r="5">
@@ -659,10 +659,10 @@
         <v>0.4021114024077352</v>
       </c>
       <c r="F5">
-        <v>95.08300676656251</v>
+        <v>110.6795104085185</v>
       </c>
       <c r="G5">
-        <v>0.1287416890915327</v>
+        <v>0.1321979250596891</v>
       </c>
       <c r="H5">
         <v>3.35</v>
@@ -700,7 +700,7 @@
         <v>0.2021585358630746</v>
       </c>
       <c r="S5">
-        <v>0.4310571780827911</v>
+        <v>0.4315509260782421</v>
       </c>
     </row>
     <row r="6">
@@ -722,10 +722,10 @@
         <v>0.2559912061846156</v>
       </c>
       <c r="F6">
-        <v>104.9201081617857</v>
+        <v>123.4828555304348</v>
       </c>
       <c r="G6">
-        <v>0.1651999633930487</v>
+        <v>0.1728636538496925</v>
       </c>
       <c r="H6">
         <v>1.864406779661017</v>
@@ -763,7 +763,7 @@
         <v>0.3020226232484428</v>
       </c>
       <c r="S6">
-        <v>0.3801502907151748</v>
+        <v>0.3812451036375524</v>
       </c>
     </row>
     <row r="7">
@@ -785,10 +785,10 @@
         <v>0.6824439679874053</v>
       </c>
       <c r="F7">
-        <v>190.1838700915625</v>
+        <v>218.0827665203704</v>
       </c>
       <c r="G7">
-        <v>0.4812045968234252</v>
+        <v>0.4733299997337918</v>
       </c>
       <c r="H7">
         <v>12.89830508474576</v>
@@ -826,7 +826,7 @@
         <v>0.7074196364968555</v>
       </c>
       <c r="S7">
-        <v>0.6023658462599593</v>
+        <v>0.6012409038185831</v>
       </c>
     </row>
     <row r="8">
@@ -848,10 +848,10 @@
         <v>0.4023952804604635</v>
       </c>
       <c r="F8">
-        <v>116.0377657446875</v>
+        <v>133.3449700559259</v>
       </c>
       <c r="G8">
-        <v>0.2064042362233141</v>
+        <v>0.2041875048254093</v>
       </c>
       <c r="H8">
         <v>2</v>
@@ -889,7 +889,7 @@
         <v>0.2737238705025282</v>
       </c>
       <c r="S8">
-        <v>0.4194639014490705</v>
+        <v>0.419147225535084</v>
       </c>
     </row>
     <row r="9">
@@ -911,10 +911,10 @@
         <v>0.3367709474237064</v>
       </c>
       <c r="F9">
-        <v>98.8683452184375</v>
+        <v>111.0446189811111</v>
       </c>
       <c r="G9">
-        <v>0.1427709139676277</v>
+        <v>0.1333575756080868</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -952,7 +952,7 @@
         <v>0.3692594182722592</v>
       </c>
       <c r="S9">
-        <v>0.3364964879525594</v>
+        <v>0.3351517253297678</v>
       </c>
     </row>
     <row r="10">
@@ -974,10 +974,10 @@
         <v>0.5836562254685655</v>
       </c>
       <c r="F10">
-        <v>119.3581357134375</v>
+        <v>137.07819946</v>
       </c>
       <c r="G10">
-        <v>0.2187101944766251</v>
+        <v>0.2160449134175649</v>
       </c>
       <c r="H10">
         <v>11.03333333333333</v>
@@ -1015,7 +1015,7 @@
         <v>0.7517332556213703</v>
       </c>
       <c r="S10">
-        <v>0.5603891394375248</v>
+        <v>0.5600083850005162</v>
       </c>
     </row>
     <row r="11">
@@ -1037,10 +1037,10 @@
         <v>0.4537123474411335</v>
       </c>
       <c r="F11">
-        <v>120.089965424375</v>
+        <v>129.6514192474074</v>
       </c>
       <c r="G11">
-        <v>0.2214225024290789</v>
+        <v>0.1924561225951354</v>
       </c>
       <c r="H11">
         <v>5.3</v>
@@ -1078,7 +1078,7 @@
         <v>0.4533593021840931</v>
       </c>
       <c r="S11">
-        <v>0.4687617659102406</v>
+        <v>0.4646237116482487</v>
       </c>
     </row>
     <row r="12">
@@ -1100,10 +1100,10 @@
         <v>0.3288492631064082</v>
       </c>
       <c r="F12">
-        <v>99.45453668906251</v>
+        <v>115.78909633</v>
       </c>
       <c r="G12">
-        <v>0.1449434573389538</v>
+        <v>0.1484268897039762</v>
       </c>
       <c r="H12">
         <v>3.2</v>
@@ -1141,7 +1141,7 @@
         <v>0.4480599402953412</v>
       </c>
       <c r="S12">
-        <v>0.4377548012351757</v>
+        <v>0.438252434430179</v>
       </c>
     </row>
     <row r="13">
@@ -1163,10 +1163,10 @@
         <v>0.6292839319183426</v>
       </c>
       <c r="F13">
-        <v>192.928677510625</v>
+        <v>223.4902612148148</v>
       </c>
       <c r="G13">
-        <v>0.4913774046220325</v>
+        <v>0.4905051762664656</v>
       </c>
       <c r="H13">
         <v>6.559322033898305</v>
@@ -1204,7 +1204,7 @@
         <v>0.7124206934329075</v>
       </c>
       <c r="S13">
-        <v>0.658513344656423</v>
+        <v>0.6583887406056277</v>
       </c>
     </row>
     <row r="14">
@@ -1226,10 +1226,10 @@
         <v>0.3531179340704553</v>
       </c>
       <c r="F14">
-        <v>67.78081792354838</v>
+        <v>79.78627797423077</v>
       </c>
       <c r="G14">
-        <v>0.02755429151588618</v>
+        <v>0.03407545787189094</v>
       </c>
       <c r="H14">
         <v>0.95</v>
@@ -1267,7 +1267,7 @@
         <v>0.3132008182870046</v>
       </c>
       <c r="S14">
-        <v>0.3778547477728379</v>
+        <v>0.3787863429665529</v>
       </c>
     </row>
     <row r="15">
@@ -1289,10 +1289,10 @@
         <v>0.4605975769010921</v>
       </c>
       <c r="F15">
-        <v>126.9768313448387</v>
+        <v>147.3560944807692</v>
       </c>
       <c r="G15">
-        <v>0.2469466112817081</v>
+        <v>0.248689358089394</v>
       </c>
       <c r="H15">
         <v>1.983050847457627</v>
@@ -1330,7 +1330,7 @@
         <v>0.6947836406760127</v>
       </c>
       <c r="S15">
-        <v>0.437165158624029</v>
+        <v>0.4374141224536984</v>
       </c>
     </row>
     <row r="16">
@@ -1352,10 +1352,10 @@
         <v>0.5304077887594206</v>
       </c>
       <c r="F16">
-        <v>184.2882473682143</v>
+        <v>218.6172393317391</v>
       </c>
       <c r="G16">
-        <v>0.4593542344259761</v>
+        <v>0.4750275815911728</v>
       </c>
       <c r="H16">
         <v>2</v>
@@ -1393,7 +1393,7 @@
         <v>0.3834795696361811</v>
       </c>
       <c r="S16">
-        <v>0.4516765065936149</v>
+        <v>0.453915556188643</v>
       </c>
     </row>
     <row r="17">
@@ -1415,10 +1415,10 @@
         <v>0.313670539220751</v>
       </c>
       <c r="F17">
-        <v>85.71637923125</v>
+        <v>98.60168228703704</v>
       </c>
       <c r="G17">
-        <v>0.09402708544534275</v>
+        <v>0.09383656886069811</v>
       </c>
       <c r="H17">
         <v>1</v>
@@ -1456,7 +1456,7 @@
         <v>0.3681243883393301</v>
       </c>
       <c r="S17">
-        <v>0.1860029160505696</v>
+        <v>0.1859756993956204</v>
       </c>
     </row>
     <row r="18">
@@ -1478,10 +1478,10 @@
         <v>0.5859329628396042</v>
       </c>
       <c r="F18">
-        <v>196.8196160846875</v>
+        <v>226.3424978181482</v>
       </c>
       <c r="G18">
-        <v>0.5057980047687795</v>
+        <v>0.4995643931392132</v>
       </c>
       <c r="H18">
         <v>3.559322033898305</v>
@@ -1519,7 +1519,7 @@
         <v>0.6150179637492951</v>
       </c>
       <c r="S18">
-        <v>0.4886782149597833</v>
+        <v>0.4877876990127024</v>
       </c>
     </row>
     <row r="19">
@@ -1541,10 +1541,10 @@
         <v>0.5679576140152887</v>
       </c>
       <c r="F19">
-        <v>123.234310468125</v>
+        <v>137.8385049933333</v>
       </c>
       <c r="G19">
-        <v>0.233076076942331</v>
+        <v>0.2184597806512183</v>
       </c>
       <c r="H19">
         <v>12.15254237288136</v>
@@ -1582,7 +1582,7 @@
         <v>0.6351893924374753</v>
       </c>
       <c r="S19">
-        <v>0.6185564065771568</v>
+        <v>0.6164683642498551</v>
       </c>
     </row>
     <row r="20">
@@ -1604,10 +1604,10 @@
         <v>0.4864250121536806</v>
       </c>
       <c r="F20">
-        <v>140.165478528125</v>
+        <v>152.6567249751852</v>
       </c>
       <c r="G20">
-        <v>0.2958263876869464</v>
+        <v>0.265525114686548</v>
       </c>
       <c r="H20">
         <v>3.694915254237288</v>
@@ -1645,7 +1645,7 @@
         <v>0.5400635442923848</v>
       </c>
       <c r="S20">
-        <v>0.4769163801276965</v>
+        <v>0.4725876268419253</v>
       </c>
     </row>
     <row r="21">
@@ -1667,10 +1667,10 @@
         <v>0.4422947815550168</v>
       </c>
       <c r="F21">
-        <v>112.8774740863333</v>
+        <v>128.430548844</v>
       </c>
       <c r="G21">
-        <v>0.1946915603522473</v>
+        <v>0.188578418429548</v>
       </c>
       <c r="H21">
         <v>3.6</v>
@@ -1708,7 +1708,7 @@
         <v>0.7200410734080649</v>
       </c>
       <c r="S21">
-        <v>0.4817210942956662</v>
+        <v>0.4808477883067092</v>
       </c>
     </row>
     <row r="22">
@@ -1730,10 +1730,10 @@
         <v>0.7410034679201478</v>
       </c>
       <c r="F22">
-        <v>195.54534427125</v>
+        <v>220.6409793874074</v>
       </c>
       <c r="G22">
-        <v>0.5010752973936624</v>
+        <v>0.481455344293937</v>
       </c>
       <c r="H22">
         <v>1.983050847457627</v>
@@ -1765,7 +1765,7 @@
         <v>0.6679926389079232</v>
       </c>
       <c r="S22">
-        <v>0.5985903479605003</v>
+        <v>0.5953203557772127</v>
       </c>
     </row>
     <row r="23">
@@ -1787,10 +1787,10 @@
         <v>0.2815616571454121</v>
       </c>
       <c r="F23">
-        <v>119.3736232370968</v>
+        <v>139.410289585</v>
       </c>
       <c r="G23">
-        <v>0.2187675943511546</v>
+        <v>0.2234520514454821</v>
       </c>
       <c r="H23">
         <v>1</v>
@@ -1828,7 +1828,7 @@
         <v>0.129348291469426</v>
       </c>
       <c r="S23">
-        <v>0.2177428250114373</v>
+        <v>0.2184120331677698</v>
       </c>
     </row>
     <row r="24">
@@ -1850,10 +1850,10 @@
         <v>0.322165014161533</v>
       </c>
       <c r="F24">
-        <v>80.2080049490625</v>
+        <v>93.11473346</v>
       </c>
       <c r="G24">
-        <v>0.07361194357916995</v>
+        <v>0.07640903170066567</v>
       </c>
       <c r="H24">
         <v>0.9833333333333333</v>
@@ -1885,7 +1885,7 @@
         <v>0.374455591094319</v>
       </c>
       <c r="S24">
-        <v>0.38742213348037</v>
+        <v>0.3878883148339526</v>
       </c>
     </row>
     <row r="25">
@@ -1907,10 +1907,10 @@
         <v>0.5210945463425779</v>
       </c>
       <c r="F25">
-        <v>123.441344703125</v>
+        <v>142.6759671048148</v>
       </c>
       <c r="G25">
-        <v>0.2338433874158308</v>
+        <v>0.233824431090945</v>
       </c>
       <c r="H25">
         <v>3.677966101694915</v>
@@ -1948,7 +1948,7 @@
         <v>0.5641299519016463</v>
       </c>
       <c r="S25">
-        <v>0.4649817286833527</v>
+        <v>0.4649790206369404</v>
       </c>
     </row>
     <row r="26">
@@ -1970,10 +1970,10 @@
         <v>0.4335613624583748</v>
       </c>
       <c r="F26">
-        <v>177.1940864143333</v>
+        <v>207.2343066116</v>
       </c>
       <c r="G26">
-        <v>0.4330618485285115</v>
+        <v>0.438873338272396</v>
       </c>
       <c r="H26">
         <v>1.627118644067797</v>
@@ -2011,7 +2011,7 @@
         <v>0.3160078826273875</v>
       </c>
       <c r="S26">
-        <v>0.3848268233136405</v>
+        <v>0.3856570361341954</v>
       </c>
     </row>
     <row r="27">
@@ -2033,10 +2033,10 @@
         <v>0.4941534023740833</v>
       </c>
       <c r="F27">
-        <v>168.7766671846875</v>
+        <v>196.5014849340741</v>
       </c>
       <c r="G27">
-        <v>0.4018652015838838</v>
+        <v>0.4047839646490428</v>
       </c>
       <c r="H27">
         <v>3.933333333333333</v>
@@ -2074,7 +2074,7 @@
         <v>0.5587002648975824</v>
       </c>
       <c r="S27">
-        <v>0.4767183428919147</v>
+        <v>0.4771353090440803</v>
       </c>
     </row>
     <row r="28">
@@ -2096,10 +2096,10 @@
         <v>0.8830837022171001</v>
       </c>
       <c r="F28">
-        <v>232.0746173662963</v>
+        <v>270.3988719609091</v>
       </c>
       <c r="G28">
-        <v>0.6364601231697685</v>
+        <v>0.6394953678415722</v>
       </c>
       <c r="H28">
         <v>12.86440677966102</v>
@@ -2137,7 +2137,7 @@
         <v>0.8774595492880565</v>
       </c>
       <c r="S28">
-        <v>0.6451374135252902</v>
+        <v>0.6455710199069764</v>
       </c>
     </row>
     <row r="29">
@@ -2159,10 +2159,10 @@
         <v>0.5780916197159226</v>
       </c>
       <c r="F29">
-        <v>164.713646173125</v>
+        <v>190.4956535322222</v>
       </c>
       <c r="G29">
-        <v>0.3868068293479019</v>
+        <v>0.3857083630292655</v>
       </c>
       <c r="H29">
         <v>6.135593220338983</v>
@@ -2200,7 +2200,7 @@
         <v>0.6528597475257988</v>
       </c>
       <c r="S29">
-        <v>0.4726451900413647</v>
+        <v>0.4724882662815595</v>
       </c>
     </row>
     <row r="30">
@@ -2222,10 +2222,10 @@
         <v>0.4821264930854841</v>
       </c>
       <c r="F30">
-        <v>93.236065658125</v>
+        <v>106.5558604737037</v>
       </c>
       <c r="G30">
-        <v>0.1218965542449143</v>
+        <v>0.1191004705837453</v>
       </c>
       <c r="H30">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         <v>0.6124200573528666</v>
       </c>
       <c r="S30">
-        <v>0.3439699751180481</v>
+        <v>0.3435705345950239</v>
       </c>
     </row>
     <row r="31">
@@ -2285,10 +2285,10 @@
         <v>0.7210649319415701</v>
       </c>
       <c r="F31">
-        <v>144.923307941875</v>
+        <v>167.819820467037</v>
       </c>
       <c r="G31">
-        <v>0.313459859466606</v>
+        <v>0.3136858354214025</v>
       </c>
       <c r="H31">
         <v>6</v>
@@ -2326,7 +2326,7 @@
         <v>0.6400236385238157</v>
       </c>
       <c r="S31">
-        <v>0.5361884341820413</v>
+        <v>0.536220716461298</v>
       </c>
     </row>
     <row r="32">
@@ -2348,10 +2348,10 @@
         <v>0.4271450080044754</v>
       </c>
       <c r="F32">
-        <v>67.318532718125</v>
+        <v>76.97403623703704</v>
       </c>
       <c r="G32">
-        <v>0.02584096965940489</v>
+        <v>0.02514327189333068</v>
       </c>
       <c r="H32">
         <v>0.7333333333333333</v>
@@ -2389,7 +2389,7 @@
         <v>0.1791742072897486</v>
       </c>
       <c r="S32">
-        <v>0.3169935983074612</v>
+        <v>0.316893927198022</v>
       </c>
     </row>
     <row r="33">
@@ -2411,10 +2411,10 @@
         <v>0.5135956637831848</v>
       </c>
       <c r="F33">
-        <v>173.841501374375</v>
+        <v>196.8053963777778</v>
       </c>
       <c r="G33">
-        <v>0.4206364947484525</v>
+        <v>0.4057492421002207</v>
       </c>
       <c r="H33">
         <v>3.610169491525424</v>
@@ -2452,7 +2452,7 @@
         <v>0.4809445889191414</v>
       </c>
       <c r="S33">
-        <v>0.4584120797393729</v>
+        <v>0.456285329361054</v>
       </c>
     </row>
     <row r="34">
@@ -2474,10 +2474,10 @@
         <v>0.6362294846750176</v>
       </c>
       <c r="F34">
-        <v>124.1271808390625</v>
+        <v>140.1377522314815</v>
       </c>
       <c r="G34">
-        <v>0.2363852339380231</v>
+        <v>0.2257626037585675</v>
       </c>
       <c r="H34">
         <v>6.220338983050848</v>
@@ -2515,7 +2515,7 @@
         <v>0.6190463355929701</v>
       </c>
       <c r="S34">
-        <v>0.5599671240568403</v>
+        <v>0.5584496054597753</v>
       </c>
     </row>
     <row r="35">
@@ -2537,10 +2537,10 @@
         <v>0.6801308891122624</v>
       </c>
       <c r="F35">
-        <v>175.416226305</v>
+        <v>200.1776174840741</v>
       </c>
       <c r="G35">
-        <v>0.4264727417447518</v>
+        <v>0.4164600233548656</v>
       </c>
       <c r="H35">
         <v>11.2</v>
@@ -2578,7 +2578,7 @@
         <v>0.6217216854641848</v>
       </c>
       <c r="S35">
-        <v>0.5107716399908507</v>
+        <v>0.5093412516494384</v>
       </c>
     </row>
     <row r="36">
@@ -2600,10 +2600,10 @@
         <v>0.5944161584257603</v>
       </c>
       <c r="F36">
-        <v>161.3252078546875</v>
+        <v>184.1943009733333</v>
       </c>
       <c r="G36">
-        <v>0.3742485961139383</v>
+        <v>0.3656941330190682</v>
       </c>
       <c r="H36">
         <v>2</v>
@@ -2641,7 +2641,7 @@
         <v>0.4683722004833799</v>
       </c>
       <c r="S36">
-        <v>0.4369903364095117</v>
+        <v>0.4357682702531017</v>
       </c>
     </row>
     <row r="37">
@@ -2663,10 +2663,10 @@
         <v>0.5277366427817703</v>
       </c>
       <c r="F37">
-        <v>125.714529449375</v>
+        <v>144.7306987062963</v>
       </c>
       <c r="G37">
-        <v>0.2422682668276714</v>
+        <v>0.2403506285218856</v>
       </c>
       <c r="H37">
         <v>1.88135593220339</v>
@@ -2704,7 +2704,7 @@
         <v>0.4727623426593815</v>
       </c>
       <c r="S37">
-        <v>0.408662718244595</v>
+        <v>0.4083887699151971</v>
       </c>
     </row>
     <row r="38">
@@ -2726,10 +2726,10 @@
         <v>0.6956075427970684</v>
       </c>
       <c r="F38">
-        <v>151.1668673634375</v>
+        <v>174.5047560962963</v>
       </c>
       <c r="G38">
-        <v>0.3365997451772152</v>
+        <v>0.3349183943104657</v>
       </c>
       <c r="H38">
         <v>6.915254237288136</v>
@@ -2767,7 +2767,7 @@
         <v>0.7131341149161409</v>
       </c>
       <c r="S38">
-        <v>0.6261942424572879</v>
+        <v>0.6259540494763237</v>
       </c>
     </row>
     <row r="39">
@@ -2789,10 +2789,10 @@
         <v>0.8210194478581516</v>
       </c>
       <c r="F39">
-        <v>181.2209807528125</v>
+        <v>208.5559138366667</v>
       </c>
       <c r="G39">
-        <v>0.4479863280552536</v>
+        <v>0.4430710007168358</v>
       </c>
       <c r="H39">
         <v>11.22033898305085</v>
@@ -2830,7 +2830,7 @@
         <v>0.6764471899547364</v>
       </c>
       <c r="S39">
-        <v>0.6370063394134295</v>
+        <v>0.6363041497936556</v>
       </c>
     </row>
     <row r="40">
@@ -2852,10 +2852,10 @@
         <v>0.4390805957391429</v>
       </c>
       <c r="F40">
-        <v>133.0338306171875</v>
+        <v>152.0955397151852</v>
       </c>
       <c r="G40">
-        <v>0.2693950675945206</v>
+        <v>0.2637426892839051</v>
       </c>
       <c r="H40">
         <v>1</v>
@@ -2893,7 +2893,7 @@
         <v>0.4996335043034948</v>
       </c>
       <c r="S40">
-        <v>0.4174890228783035</v>
+        <v>0.4166815402625013</v>
       </c>
     </row>
     <row r="41">
@@ -2915,10 +2915,10 @@
         <v>0.2968748841847817</v>
       </c>
       <c r="F41">
-        <v>108.986184225625</v>
+        <v>127.1470300633333</v>
       </c>
       <c r="G41">
-        <v>0.1802696582666082</v>
+        <v>0.1845017317406826</v>
       </c>
       <c r="H41">
         <v>1.932203389830508</v>
@@ -2956,7 +2956,7 @@
         <v>0.4603998087123266</v>
       </c>
       <c r="S41">
-        <v>0.3265993546361881</v>
+        <v>0.3272039365610559</v>
       </c>
     </row>
     <row r="42">
@@ -2978,10 +2978,10 @@
         <v>0.5122807381847606</v>
       </c>
       <c r="F42">
-        <v>119.8886665934375</v>
+        <v>137.3126007962963</v>
       </c>
       <c r="G42">
-        <v>0.2206764485154273</v>
+        <v>0.2167894142553594</v>
       </c>
       <c r="H42">
         <v>3.491525423728814</v>
@@ -3019,7 +3019,7 @@
         <v>0.4549699493610279</v>
       </c>
       <c r="S42">
-        <v>0.4827249565776124</v>
+        <v>0.4821696659690312</v>
       </c>
     </row>
     <row r="43">
@@ -3041,10 +3041,10 @@
         <v>0.5475455574012923</v>
       </c>
       <c r="F43">
-        <v>155.2948253259375</v>
+        <v>177.0335387388889</v>
       </c>
       <c r="G43">
-        <v>0.3518987868009025</v>
+        <v>0.3429502631801497</v>
       </c>
       <c r="H43">
         <v>6.35593220338983</v>
@@ -3076,7 +3076,7 @@
         <v>0.7769677965397922</v>
       </c>
       <c r="S43">
-        <v>0.4976488390422292</v>
+        <v>0.4961574184387704</v>
       </c>
     </row>
     <row r="44">
@@ -3098,10 +3098,10 @@
         <v>0.6505704254947626</v>
       </c>
       <c r="F44">
-        <v>112.6675989174194</v>
+        <v>128.5063440026923</v>
       </c>
       <c r="G44">
-        <v>0.1939137208068444</v>
+        <v>0.188819157497161</v>
       </c>
       <c r="H44">
         <v>5.491525423728813</v>
@@ -3139,7 +3139,7 @@
         <v>0.7131434838109965</v>
       </c>
       <c r="S44">
-        <v>0.5514051765935161</v>
+        <v>0.5506773818349899</v>
       </c>
     </row>
     <row r="45">
@@ -3161,10 +3161,10 @@
         <v>0.6028230402012745</v>
       </c>
       <c r="F45">
-        <v>202.9518392865625</v>
+        <v>233.8890457351852</v>
       </c>
       <c r="G45">
-        <v>0.5285252560788698</v>
+        <v>0.5235335877498996</v>
       </c>
       <c r="H45">
         <v>1</v>
@@ -3196,7 +3196,7 @@
         <v>0.5477830485890927</v>
       </c>
       <c r="S45">
-        <v>0.6561743309314412</v>
+        <v>0.6553423862099461</v>
       </c>
     </row>
     <row r="46">
@@ -3218,10 +3218,10 @@
         <v>0.5537858828691359</v>
       </c>
       <c r="F46">
-        <v>107.9302736590323</v>
+        <v>113.04228152</v>
       </c>
       <c r="G46">
-        <v>0.1763562415467805</v>
+        <v>0.1397025114234424</v>
       </c>
       <c r="H46">
         <v>6.203389830508475</v>
@@ -3259,7 +3259,7 @@
         <v>0.4893672453337708</v>
       </c>
       <c r="S46">
-        <v>0.5605146775977388</v>
+        <v>0.5552784304372619</v>
       </c>
     </row>
     <row r="47">
@@ -3281,10 +3281,10 @@
         <v>0.4184983987891018</v>
       </c>
       <c r="F47">
-        <v>115.11182788125</v>
+        <v>131.2954112092593</v>
       </c>
       <c r="G47">
-        <v>0.2029725244562933</v>
+        <v>0.1976777369948891</v>
       </c>
       <c r="H47">
         <v>1.864406779661017</v>
@@ -3316,7 +3316,7 @@
         <v>0.3514288875039369</v>
       </c>
       <c r="S47">
-        <v>0.4000617457049202</v>
+        <v>0.3991792811280195</v>
       </c>
     </row>
     <row r="48">
@@ -3338,10 +3338,10 @@
         <v>0.6881147050334921</v>
       </c>
       <c r="F48">
-        <v>254.4268867953125</v>
+        <v>288.1408273914815</v>
       </c>
       <c r="G48">
-        <v>0.7193021248289343</v>
+        <v>0.6958470119528418</v>
       </c>
       <c r="H48">
         <v>11.5</v>
@@ -3373,7 +3373,7 @@
         <v>0.8875126067532404</v>
       </c>
       <c r="S48">
-        <v>0.7069031037108603</v>
+        <v>0.7029939182315115</v>
       </c>
     </row>
     <row r="49">
@@ -3395,10 +3395,10 @@
         <v>0.5647279988701689</v>
       </c>
       <c r="F49">
-        <v>231.912202086875</v>
+        <v>260.7046894659259</v>
       </c>
       <c r="G49">
-        <v>0.635858179510758</v>
+        <v>0.6087048992235723</v>
       </c>
       <c r="H49">
         <v>3.254237288135593</v>
@@ -3436,7 +3436,7 @@
         <v>0.9804228446434465</v>
       </c>
       <c r="S49">
-        <v>0.5218447535011101</v>
+        <v>0.5179657134600837</v>
       </c>
     </row>
     <row r="50">
@@ -3458,10 +3458,10 @@
         <v>0.3551590788297286</v>
       </c>
       <c r="F50">
-        <v>115.4052684690625</v>
+        <v>134.3678353466667</v>
       </c>
       <c r="G50">
-        <v>0.2040600742346113</v>
+        <v>0.2074363091109994</v>
       </c>
       <c r="H50">
         <v>1</v>
@@ -3499,7 +3499,7 @@
         <v>0.4722015136365176</v>
       </c>
       <c r="S50">
-        <v>0.3708611723194072</v>
+        <v>0.3713434915874627</v>
       </c>
     </row>
     <row r="51">
@@ -3521,10 +3521,10 @@
         <v>0.6509749520708715</v>
       </c>
       <c r="F51">
-        <v>268.7253422890625</v>
+        <v>300.0112017037037</v>
       </c>
       <c r="G51">
-        <v>0.7722950738222517</v>
+        <v>0.7335494575106325</v>
       </c>
       <c r="H51">
         <v>3.033898305084746</v>
@@ -3556,7 +3556,7 @@
         <v>0.8661985237387249</v>
       </c>
       <c r="S51">
-        <v>0.6420613476676871</v>
+        <v>0.6356037449490839</v>
       </c>
     </row>
     <row r="52">
@@ -3578,10 +3578,10 @@
         <v>0.5761905996751149</v>
       </c>
       <c r="F52">
-        <v>102.683986036875</v>
+        <v>111.8974685614815</v>
       </c>
       <c r="G52">
-        <v>0.1569124455027409</v>
+        <v>0.1360663793936414</v>
       </c>
       <c r="H52">
         <v>10.33898305084746</v>
@@ -3619,7 +3619,7 @@
         <v>0.6543190589226516</v>
       </c>
       <c r="S52">
-        <v>0.5019408141296289</v>
+        <v>0.4989628046854718</v>
       </c>
     </row>
     <row r="53">
@@ -3641,10 +3641,10 @@
         <v>0.3200677323665221</v>
       </c>
       <c r="F53">
-        <v>89.29260579419355</v>
+        <v>103.3193545726923</v>
       </c>
       <c r="G53">
-        <v>0.107281299645013</v>
+        <v>0.1088207452506773</v>
       </c>
       <c r="H53">
         <v>1</v>
@@ -3682,7 +3682,7 @@
         <v>0.2300217547418851</v>
       </c>
       <c r="S53">
-        <v>0.338697663862537</v>
+        <v>0.3389175846633461</v>
       </c>
     </row>
     <row r="54">
@@ -3704,10 +3704,10 @@
         <v>0.4395619186599191</v>
       </c>
       <c r="F54">
-        <v>118.3972807875</v>
+        <v>136.8585653651852</v>
       </c>
       <c r="G54">
-        <v>0.2151490730602286</v>
+        <v>0.215347315996912</v>
       </c>
       <c r="H54">
         <v>1.983050847457627</v>
@@ -3745,7 +3745,7 @@
         <v>0.6549505545122504</v>
       </c>
       <c r="S54">
-        <v>0.3695520298920587</v>
+        <v>0.3695803503115849</v>
       </c>
     </row>
     <row r="55">
@@ -3767,10 +3767,10 @@
         <v>0.5408875110612112</v>
       </c>
       <c r="F55">
-        <v>151.9766271153571</v>
+        <v>181.0067190926087</v>
       </c>
       <c r="G55">
-        <v>0.3396008775197312</v>
+        <v>0.3555697991810629</v>
       </c>
       <c r="H55">
         <v>5.186440677966102</v>
@@ -3808,7 +3808,7 @@
         <v>0.6025622161214722</v>
       </c>
       <c r="S55">
-        <v>0.6394172148449796</v>
+        <v>0.641698489368027</v>
       </c>
     </row>
     <row r="56">
@@ -3830,10 +3830,10 @@
         <v>0.5493283902064392</v>
       </c>
       <c r="F56">
-        <v>143.5188982909375</v>
+        <v>167.4246362551852</v>
       </c>
       <c r="G56">
-        <v>0.3082548351176205</v>
+        <v>0.3124306592289128</v>
       </c>
       <c r="H56">
         <v>1.983050847457627</v>
@@ -3871,7 +3871,7 @@
         <v>0.4681075174785018</v>
       </c>
       <c r="S56">
-        <v>0.5292033314007514</v>
+        <v>0.5297998777023646</v>
       </c>
     </row>
     <row r="57">
@@ -3893,10 +3893,10 @@
         <v>0.7718758408691314</v>
       </c>
       <c r="F57">
-        <v>183.8040500878125</v>
+        <v>209.0077917292593</v>
       </c>
       <c r="G57">
-        <v>0.4575597020169162</v>
+        <v>0.4445062462445779</v>
       </c>
       <c r="H57">
         <v>12.3</v>
@@ -3934,7 +3934,7 @@
         <v>1</v>
       </c>
       <c r="S57">
-        <v>0.7221078720394447</v>
+        <v>0.7202430926433964</v>
       </c>
     </row>
     <row r="58">
@@ -3956,10 +3956,10 @@
         <v>0.7184684060747184</v>
       </c>
       <c r="F58">
-        <v>117.7899405009375</v>
+        <v>137.6317868540741</v>
       </c>
       <c r="G58">
-        <v>0.2128981479276881</v>
+        <v>0.2178032066303633</v>
       </c>
       <c r="H58">
         <v>3.416666666666667</v>
@@ -3997,7 +3997,7 @@
         <v>0.7193375451729008</v>
       </c>
       <c r="S58">
-        <v>0.592461695362043</v>
+        <v>0.5931624180338537</v>
       </c>
     </row>
     <row r="59">
@@ -4019,10 +4019,10 @@
         <v>0.5900632347324082</v>
       </c>
       <c r="F59">
-        <v>134.8362436684375</v>
+        <v>155.1610474259259</v>
       </c>
       <c r="G59">
-        <v>0.2760751725143514</v>
+        <v>0.2734792935839217</v>
       </c>
       <c r="H59">
         <v>11.28813559322034</v>
@@ -4060,7 +4060,7 @@
         <v>0.8052804788124337</v>
       </c>
       <c r="S59">
-        <v>0.6274211676974397</v>
+        <v>0.6270503278502354</v>
       </c>
     </row>
     <row r="60">
@@ -4082,10 +4082,10 @@
         <v>0.6853782943919974</v>
       </c>
       <c r="F60">
-        <v>200.0871802265625</v>
+        <v>229.7353989774074</v>
       </c>
       <c r="G60">
-        <v>0.5179082540176206</v>
+        <v>0.5103408579646083</v>
       </c>
       <c r="H60">
         <v>13</v>
@@ -4123,7 +4123,7 @@
         <v>0.8439022288162242</v>
       </c>
       <c r="S60">
-        <v>0.5982398362383838</v>
+        <v>0.597158779659382</v>
       </c>
     </row>
     <row r="61">
@@ -4145,10 +4145,10 @@
         <v>1</v>
       </c>
       <c r="F61">
-        <v>146.71501500875</v>
+        <v>169.0143546955556</v>
       </c>
       <c r="G61">
-        <v>0.3201002858572309</v>
+        <v>0.3174798911548654</v>
       </c>
       <c r="H61">
         <v>2.95</v>
@@ -4186,7 +4186,7 @@
         <v>0.6007583638026363</v>
       </c>
       <c r="S61">
-        <v>0.5029674549310557</v>
+        <v>0.5025931128307177</v>
       </c>
     </row>
     <row r="62">
@@ -4208,10 +4208,10 @@
         <v>0.4822341256760957</v>
       </c>
       <c r="F62">
-        <v>190.33094006125</v>
+        <v>213.8371436925926</v>
       </c>
       <c r="G62">
-        <v>0.4817496676812886</v>
+        <v>0.4598451373939084</v>
       </c>
       <c r="H62">
         <v>7.689655172413793</v>
@@ -4249,7 +4249,7 @@
         <v>0.6577200663611824</v>
       </c>
       <c r="S62">
-        <v>0.4791251727646829</v>
+        <v>0.4759959541522</v>
       </c>
     </row>
     <row r="63">
@@ -4271,10 +4271,10 @@
         <v>0.3671409097550509</v>
       </c>
       <c r="F63">
-        <v>68.9591740921875</v>
+        <v>79.62046578629629</v>
       </c>
       <c r="G63">
-        <v>0.03192151623942003</v>
+        <v>0.0335488085157724</v>
       </c>
       <c r="H63">
         <v>2.694915254237288</v>
@@ -4312,7 +4312,7 @@
         <v>0.271727309955794</v>
       </c>
       <c r="S63">
-        <v>0.413397701812141</v>
+        <v>0.4136301721373342</v>
       </c>
     </row>
     <row r="64">
@@ -4334,10 +4334,10 @@
         <v>0.5977681191734737</v>
       </c>
       <c r="F64">
-        <v>154.55160473125</v>
+        <v>178.3186385296296</v>
       </c>
       <c r="G64">
-        <v>0.3491442619445448</v>
+        <v>0.3470319714416021</v>
       </c>
       <c r="H64">
         <v>6.677966101694915</v>
@@ -4375,7 +4375,7 @@
         <v>0.578059215922415</v>
       </c>
       <c r="S64">
-        <v>0.4295432909397365</v>
+        <v>0.4292415351536018</v>
       </c>
     </row>
     <row r="65">
@@ -4397,10 +4397,10 @@
         <v>0.5363960821200183</v>
       </c>
       <c r="F65">
-        <v>73.60762752531249</v>
+        <v>85.41424579185185</v>
       </c>
       <c r="G65">
-        <v>0.04914961865838969</v>
+        <v>0.05195089673032519</v>
       </c>
       <c r="H65">
         <v>1</v>
@@ -4438,7 +4438,7 @@
         <v>0.2024667529990534</v>
       </c>
       <c r="S65">
-        <v>0.4907230701504024</v>
+        <v>0.4911232527321074</v>
       </c>
     </row>
     <row r="66">
@@ -4460,7 +4460,7 @@
         <v>0.7780287209137213</v>
       </c>
       <c r="F66">
-        <v>330.164247171875</v>
+        <v>383.901454132963</v>
       </c>
       <c r="G66">
         <v>1</v>
@@ -4523,10 +4523,10 @@
         <v>0.4488973724545661</v>
       </c>
       <c r="F67">
-        <v>76.5980043496875</v>
+        <v>89.07657681111111</v>
       </c>
       <c r="G67">
-        <v>0.06023255601439794</v>
+        <v>0.06358311929015284</v>
       </c>
       <c r="H67">
         <v>3.779661016949153</v>
@@ -4564,7 +4564,7 @@
         <v>0.3929600629229978</v>
       </c>
       <c r="S67">
-        <v>0.4601836628180562</v>
+        <v>0.4606623147145926</v>
       </c>
     </row>
     <row r="68">
@@ -4586,10 +4586,10 @@
         <v>0.5051754831240297</v>
       </c>
       <c r="F68">
-        <v>162.0354838759375</v>
+        <v>190.2813164281481</v>
       </c>
       <c r="G68">
-        <v>0.3768810217617106</v>
+        <v>0.385027589804697</v>
       </c>
       <c r="H68">
         <v>0.9833333333333333</v>
@@ -4621,7 +4621,7 @@
         <v>0.3671890722886557</v>
       </c>
       <c r="S68">
-        <v>0.4008122997475896</v>
+        <v>0.4021700610880873</v>
       </c>
     </row>
     <row r="69">
@@ -4643,10 +4643,10 @@
         <v>0.3379120036940255</v>
       </c>
       <c r="F69">
-        <v>88.9824012521875</v>
+        <v>103.6936781292593</v>
       </c>
       <c r="G69">
-        <v>0.1061316192841371</v>
+        <v>0.1100096642469328</v>
       </c>
       <c r="H69">
         <v>0.9833333333333333</v>
@@ -4684,7 +4684,7 @@
         <v>0</v>
       </c>
       <c r="S69">
-        <v>0.3102788828933085</v>
+        <v>0.310832889316565</v>
       </c>
     </row>
     <row r="70">
@@ -4706,10 +4706,10 @@
         <v>0.5803707375306559</v>
       </c>
       <c r="F70">
-        <v>102.4966450978125</v>
+        <v>117.7034853077778</v>
       </c>
       <c r="G70">
-        <v>0.1562181223408834</v>
+        <v>0.1545073336994773</v>
       </c>
       <c r="H70">
         <v>2</v>
@@ -4747,7 +4747,7 @@
         <v>0.3555699805594751</v>
       </c>
       <c r="S70">
-        <v>0.4007582644216341</v>
+        <v>0.4005138660442904</v>
       </c>
     </row>
     <row r="71">
@@ -4769,7 +4769,7 @@
         <v>0.53293275740635</v>
       </c>
       <c r="F71">
-        <v>60.3461720246875</v>
+        <v>69.05783758222222</v>
       </c>
       <c r="G71">
         <v>0</v>
@@ -4832,10 +4832,10 @@
         <v>0.6040955263600328</v>
       </c>
       <c r="F72">
-        <v>135.46246887375</v>
+        <v>157.4820688440741</v>
       </c>
       <c r="G72">
-        <v>0.2783960889502532</v>
+        <v>0.2808512754064405</v>
       </c>
       <c r="H72">
         <v>6.35593220338983</v>
@@ -4873,7 +4873,7 @@
         <v>0.3793248757832806</v>
       </c>
       <c r="S72">
-        <v>0.4199460195376425</v>
+        <v>0.420296760459955</v>
       </c>
     </row>
     <row r="73">
@@ -4895,10 +4895,10 @@
         <v>0.38750825476394</v>
       </c>
       <c r="F73">
-        <v>104.8937559309375</v>
+        <v>120.6028010485185</v>
       </c>
       <c r="G73">
-        <v>0.1651022967306731</v>
+        <v>0.1637160823871721</v>
       </c>
       <c r="H73">
         <v>2</v>
@@ -4936,7 +4936,7 @@
         <v>0.197913378030515</v>
       </c>
       <c r="S73">
-        <v>0.436978979551457</v>
+        <v>0.4367809489309569</v>
       </c>
     </row>
     <row r="74">
@@ -4958,10 +4958,10 @@
         <v>0.7138177781831853</v>
       </c>
       <c r="F74">
-        <v>151.39790363125</v>
+        <v>174.2625411192593</v>
       </c>
       <c r="G74">
-        <v>0.337456012006954</v>
+        <v>0.334149075943174</v>
       </c>
       <c r="H74">
         <v>10.48333333333333</v>
@@ -4999,7 +4999,7 @@
         <v>0.5299726939760873</v>
       </c>
       <c r="S74">
-        <v>0.5770790759279339</v>
+        <v>0.5766066564902511</v>
       </c>
     </row>
     <row r="75">
@@ -5021,10 +5021,10 @@
         <v>0.6468651507261209</v>
       </c>
       <c r="F75">
-        <v>152.0578600525</v>
+        <v>174.0390576866667</v>
       </c>
       <c r="G75">
-        <v>0.3399019431066032</v>
+        <v>0.3334392523328339</v>
       </c>
       <c r="H75">
         <v>9.85</v>
@@ -5062,7 +5062,7 @@
         <v>0.410284121339076</v>
       </c>
       <c r="S75">
-        <v>0.5471463558572585</v>
+        <v>0.5462231143181486</v>
       </c>
     </row>
     <row r="76">
@@ -5084,10 +5084,10 @@
         <v>0.4296548459987961</v>
       </c>
       <c r="F76">
-        <v>61.79041457875</v>
+        <v>71.08605455481481</v>
       </c>
       <c r="G76">
-        <v>0.005352653091438228</v>
+        <v>0.006441982196789171</v>
       </c>
       <c r="H76">
         <v>1.9</v>
@@ -5125,7 +5125,7 @@
         <v>0.02939815742536144</v>
       </c>
       <c r="S76">
-        <v>0.2863759542326691</v>
+        <v>0.2865315726762906</v>
       </c>
     </row>
     <row r="77">
@@ -5147,10 +5147,10 @@
         <v>0.4584096699584418</v>
       </c>
       <c r="F77">
-        <v>114.1203750196875</v>
+        <v>127.5183824903704</v>
       </c>
       <c r="G77">
-        <v>0.1992980009425456</v>
+        <v>0.1856812138947291</v>
       </c>
       <c r="H77">
         <v>2.833333333333333</v>
@@ -5188,7 +5188,7 @@
         <v>0.6678280125044722</v>
       </c>
       <c r="S77">
-        <v>0.5230042136491669</v>
+        <v>0.5210589583566217</v>
       </c>
     </row>
     <row r="78">
@@ -5213,7 +5213,7 @@
         <v>214.3728571428572</v>
       </c>
       <c r="G78">
-        <v>0.5708538430353383</v>
+        <v>0.4615466597437452</v>
       </c>
       <c r="H78">
         <v>0.9523809523809523</v>
@@ -5227,7 +5227,7 @@
         <v>1</v>
       </c>
       <c r="S78">
-        <v>0.617095948842703</v>
+        <v>0.5806602210788387</v>
       </c>
     </row>
     <row r="79">

</xml_diff>